<commit_message>
Restrict Cozy Fantasy / Hopepunk flags to genuine genre fits
Previously these were marked Yes for any work with a hopeful tone or
cozy feeling. Tightened to: does the work actually belong to that
specific genre movement (real acknowledged darkness + hope maintained
as deliberate resistance/practice), not just have a happy ending.
Changed 41 of 46 prior Yes flags to No. These columns aren't referenced
by any score/tier formula, so no Calculated Score or tier changed.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -168,33 +168,36 @@
     <t xml:space="preserve">Studio Ghibli / Hayao Miyazaki</t>
   </si>
   <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Everyday kindness, family care and healing dominate the worldview.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiki's Delivery Service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low-stakes crisis resolved through community and personal growth.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponyo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Danger exists, but wonder, love and reconciliation remain central.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legends &amp; Lattes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travis Baldree</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
-    <t xml:space="preserve">Everyday kindness, family care and healing dominate the worldview.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kiki's Delivery Service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low-stakes crisis resolved through community and personal growth.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ponyo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Danger exists, but wonder, love and reconciliation remain central.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legends &amp; Lattes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Novel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Travis Baldree</t>
-  </si>
-  <si>
     <t xml:space="preserve">A flagship cozy fantasy built around community and second chances.</t>
   </si>
   <si>
@@ -202,9 +205,6 @@
   </si>
   <si>
     <t xml:space="preserve">T. J. Klune</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No</t>
   </si>
   <si>
     <t xml:space="preserve">Institutional prejudice is real, but empathy and care can reform lives.</t>
@@ -2184,11 +2184,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="43734253"/>
-        <c:axId val="44364566"/>
+        <c:axId val="11588857"/>
+        <c:axId val="4628358"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="43734253"/>
+        <c:axId val="11588857"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2233,7 +2233,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44364566"/>
+        <c:crossAx val="4628358"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2241,7 +2241,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44364566"/>
+        <c:axId val="4628358"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2286,7 +2286,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43734253"/>
+        <c:crossAx val="11588857"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2543,9 +2543,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>609480</xdr:colOff>
+      <xdr:colOff>609120</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>188640</xdr:rowOff>
+      <xdr:rowOff>188280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2554,7 +2554,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4890240" cy="3427200"/>
+        <a:ext cx="4889880" cy="3426840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3378,7 +3378,7 @@
         <v>56</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>48</v>
@@ -3417,7 +3417,7 @@
         <v>1</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3428,19 +3428,19 @@
         <v>27</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>55</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="H6" s="8" t="n">
         <v>0.45</v>
@@ -3496,10 +3496,10 @@
         <v>63</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="H7" s="8" t="n">
         <v>0.45</v>
@@ -3555,10 +3555,10 @@
         <v>63</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="H8" s="8" t="n">
         <v>0.45</v>
@@ -3614,7 +3614,7 @@
         <v>69</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>48</v>
@@ -3673,7 +3673,7 @@
         <v>72</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>48</v>
@@ -3732,7 +3732,7 @@
         <v>76</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>48</v>
@@ -3791,7 +3791,7 @@
         <v>76</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>48</v>
@@ -3850,7 +3850,7 @@
         <v>82</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>48</v>
@@ -3909,7 +3909,7 @@
         <v>47</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>48</v>
@@ -3968,7 +3968,7 @@
         <v>47</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>48</v>
@@ -4027,7 +4027,7 @@
         <v>90</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>48</v>
@@ -4086,7 +4086,7 @@
         <v>94</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>48</v>
@@ -4145,7 +4145,7 @@
         <v>97</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>48</v>
@@ -4204,10 +4204,10 @@
         <v>101</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="H19" s="8" t="n">
         <v>0.85</v>
@@ -4263,7 +4263,7 @@
         <v>105</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>48</v>
@@ -4322,7 +4322,7 @@
         <v>109</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>48</v>
@@ -4381,7 +4381,7 @@
         <v>113</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>48</v>
@@ -4440,7 +4440,7 @@
         <v>117</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>48</v>
@@ -4499,7 +4499,7 @@
         <v>47</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>48</v>
@@ -4558,7 +4558,7 @@
         <v>47</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>48</v>
@@ -4617,7 +4617,7 @@
         <v>82</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>48</v>
@@ -4676,7 +4676,7 @@
         <v>90</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>48</v>
@@ -4735,7 +4735,7 @@
         <v>90</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>48</v>
@@ -4794,7 +4794,7 @@
         <v>131</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>48</v>
@@ -4853,7 +4853,7 @@
         <v>76</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>48</v>
@@ -4912,7 +4912,7 @@
         <v>76</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>48</v>
@@ -4971,7 +4971,7 @@
         <v>139</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G32" s="3" t="s">
         <v>48</v>
@@ -5030,7 +5030,7 @@
         <v>142</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G33" s="3" t="s">
         <v>48</v>
@@ -5089,10 +5089,10 @@
         <v>145</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H34" s="8" t="n">
         <v>1.25</v>
@@ -5148,7 +5148,7 @@
         <v>148</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>48</v>
@@ -5207,7 +5207,7 @@
         <v>148</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>48</v>
@@ -5266,10 +5266,10 @@
         <v>82</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H37" s="8" t="n">
         <v>1.55</v>
@@ -5325,10 +5325,10 @@
         <v>156</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H38" s="8" t="n">
         <v>1.25</v>
@@ -5384,7 +5384,7 @@
         <v>160</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>48</v>
@@ -5443,7 +5443,7 @@
         <v>163</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>48</v>
@@ -5502,10 +5502,10 @@
         <v>76</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H41" s="8" t="n">
         <v>1.25</v>
@@ -5561,10 +5561,10 @@
         <v>76</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H42" s="8" t="n">
         <v>1.4</v>
@@ -5620,7 +5620,7 @@
         <v>76</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>48</v>
@@ -5679,10 +5679,10 @@
         <v>173</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H44" s="8" t="n">
         <v>1.25</v>
@@ -5738,7 +5738,7 @@
         <v>148</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>48</v>
@@ -5797,10 +5797,10 @@
         <v>179</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="H46" s="8" t="n">
         <v>1.25</v>
@@ -5856,7 +5856,7 @@
         <v>47</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>48</v>
@@ -5915,10 +5915,10 @@
         <v>184</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H48" s="8" t="n">
         <v>1.25</v>
@@ -5974,7 +5974,7 @@
         <v>187</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>48</v>
@@ -6033,7 +6033,7 @@
         <v>190</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>48</v>
@@ -6092,10 +6092,10 @@
         <v>101</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H51" s="8" t="n">
         <v>1.25</v>
@@ -6151,7 +6151,7 @@
         <v>196</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>48</v>
@@ -6210,10 +6210,10 @@
         <v>47</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H53" s="8" t="n">
         <v>1.25</v>
@@ -6269,10 +6269,10 @@
         <v>201</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H54" s="8" t="n">
         <v>1.85</v>
@@ -6328,10 +6328,10 @@
         <v>204</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H55" s="8" t="n">
         <v>1.85</v>
@@ -6387,10 +6387,10 @@
         <v>90</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H56" s="8" t="n">
         <v>2</v>
@@ -6446,10 +6446,10 @@
         <v>156</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H57" s="8" t="n">
         <v>1.7</v>
@@ -6505,10 +6505,10 @@
         <v>90</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H58" s="8" t="n">
         <v>1.9</v>
@@ -6564,10 +6564,10 @@
         <v>160</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H59" s="8" t="n">
         <v>1.95</v>
@@ -6623,10 +6623,10 @@
         <v>217</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H60" s="8" t="n">
         <v>1.95</v>
@@ -6682,10 +6682,10 @@
         <v>220</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H61" s="8" t="n">
         <v>1.9</v>
@@ -6741,10 +6741,10 @@
         <v>223</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H62" s="8" t="n">
         <v>1.7</v>
@@ -6800,10 +6800,10 @@
         <v>226</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H63" s="8" t="n">
         <v>2.4</v>
@@ -6859,10 +6859,10 @@
         <v>160</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H64" s="8" t="n">
         <v>2.2</v>
@@ -6918,10 +6918,10 @@
         <v>232</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H65" s="8" t="n">
         <v>2.2</v>
@@ -6977,10 +6977,10 @@
         <v>235</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H66" s="8" t="n">
         <v>2.35</v>
@@ -7036,10 +7036,10 @@
         <v>239</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H67" s="8" t="n">
         <v>2.2</v>
@@ -7095,10 +7095,10 @@
         <v>243</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H68" s="8" t="n">
         <v>2.95</v>
@@ -7154,10 +7154,10 @@
         <v>246</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H69" s="8" t="n">
         <v>3.2</v>
@@ -7213,10 +7213,10 @@
         <v>249</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H70" s="8" t="n">
         <v>3.5</v>
@@ -7272,10 +7272,10 @@
         <v>252</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H71" s="8" t="n">
         <v>3.2</v>
@@ -7331,10 +7331,10 @@
         <v>255</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H72" s="8" t="n">
         <v>3.2</v>
@@ -7390,10 +7390,10 @@
         <v>258</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H73" s="8" t="n">
         <v>3.6</v>
@@ -7449,10 +7449,10 @@
         <v>262</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H74" s="8" t="n">
         <v>4</v>
@@ -7508,10 +7508,10 @@
         <v>266</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H75" s="1" t="n">
         <v>0.3</v>

</xml_diff>

<commit_message>
Restore Hopepunk=Yes for the four Gentle Hopepunk (tier 1) works
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -171,6 +171,9 @@
     <t xml:space="preserve">No</t>
   </si>
   <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Everyday kindness, family care and healing dominate the worldview.</t>
   </si>
   <si>
@@ -193,9 +196,6 @@
   </si>
   <si>
     <t xml:space="preserve">Travis Baldree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes</t>
   </si>
   <si>
     <t xml:space="preserve">A flagship cozy fantasy built around community and second chances.</t>
@@ -2184,11 +2184,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="11588857"/>
-        <c:axId val="4628358"/>
+        <c:axId val="38617452"/>
+        <c:axId val="75355639"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="11588857"/>
+        <c:axId val="38617452"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2233,7 +2233,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4628358"/>
+        <c:crossAx val="75355639"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2241,7 +2241,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="4628358"/>
+        <c:axId val="75355639"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2286,7 +2286,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11588857"/>
+        <c:crossAx val="38617452"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2543,9 +2543,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>609120</xdr:colOff>
+      <xdr:colOff>608760</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>188280</xdr:rowOff>
+      <xdr:rowOff>187920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2554,7 +2554,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4889880" cy="3426840"/>
+        <a:ext cx="4889520" cy="3426480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3204,7 +3204,7 @@
         <v>48</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H2" s="8" t="n">
         <v>0.1</v>
@@ -3240,7 +3240,7 @@
         <v>1</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3251,7 +3251,7 @@
         <v>26</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>46</v>
@@ -3263,7 +3263,7 @@
         <v>48</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H3" s="8" t="n">
         <v>0.2</v>
@@ -3299,7 +3299,7 @@
         <v>1</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3310,7 +3310,7 @@
         <v>26</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>46</v>
@@ -3322,7 +3322,7 @@
         <v>48</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H4" s="8" t="n">
         <v>0.1</v>
@@ -3358,7 +3358,7 @@
         <v>1</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3369,19 +3369,19 @@
         <v>26</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H5" s="8" t="n">
         <v>0.1</v>
@@ -3431,7 +3431,7 @@
         <v>59</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>60</v>
@@ -3440,7 +3440,7 @@
         <v>48</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="H6" s="8" t="n">
         <v>0.45</v>
@@ -3490,7 +3490,7 @@
         <v>62</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>63</v>
@@ -3499,7 +3499,7 @@
         <v>48</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="H7" s="8" t="n">
         <v>0.45</v>
@@ -3549,7 +3549,7 @@
         <v>65</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>63</v>
@@ -3558,7 +3558,7 @@
         <v>48</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="H8" s="8" t="n">
         <v>0.45</v>
@@ -4207,7 +4207,7 @@
         <v>48</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="H19" s="8" t="n">
         <v>0.85</v>
@@ -5083,7 +5083,7 @@
         <v>144</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>145</v>
@@ -5142,7 +5142,7 @@
         <v>147</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>148</v>
@@ -5800,7 +5800,7 @@
         <v>48</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="H46" s="8" t="n">
         <v>1.25</v>

</xml_diff>

<commit_message>
Add Frieren to Bittersweet Hopepunk (confirmed: kindness-as-legacy, choosing connection despite certain future loss)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -2184,11 +2184,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="38617452"/>
-        <c:axId val="75355639"/>
+        <c:axId val="71486027"/>
+        <c:axId val="26757166"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="38617452"/>
+        <c:axId val="71486027"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2233,7 +2233,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75355639"/>
+        <c:crossAx val="26757166"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2241,7 +2241,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75355639"/>
+        <c:axId val="26757166"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2286,7 +2286,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38617452"/>
+        <c:crossAx val="71486027"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2543,9 +2543,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>608760</xdr:colOff>
+      <xdr:colOff>608400</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>187920</xdr:rowOff>
+      <xdr:rowOff>187560</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2554,7 +2554,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4889520" cy="3426480"/>
+        <a:ext cx="4889160" cy="3426120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4797,7 +4797,7 @@
         <v>48</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H29" s="8" t="n">
         <v>0.95</v>

</xml_diff>

<commit_message>
Document Cozy Fantasy / Hopepunk as descriptive-only tags
Confirmed: these columns stay excluded from the score formula. Wrote
up the three Hopepunk variants (Gentle/Fierce/Bittersweet) and the
Cozy Fantasy bar in both the xlsx Methodology sheet and
ADDITIONS_LOG.md so future sessions don't have to re-derive this.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="284">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -130,6 +130,45 @@
   </si>
   <si>
     <t xml:space="preserve">Very Extreme Grimdark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cozy Fantasy / Hopepunk columns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descriptive tags only -- excluded from the Weighted Internal Score / Calculated Score formula on purpose. Genre stance toward darkness is not the same as amount of darkness (e.g. Avatar: The Last Airbender is tagged Hopepunk but depicts real war and genocide).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cozy Fantasy = Yes requires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genuinely part of that specific book-publishing genre movement (comfort-focused, low-stakes, community/found-family), not just "has a cozy feeling."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hopepunk = Yes requires one of three variants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Gentle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No real adversity needed -- kindness/community/anti-cynicism as the default, deliberately-valued state of the world (e.g. Totoro, Legends &amp; Lattes).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Fierce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real external/societal adversity (an oppressive system, empire, institution) + hope/kindness as active resistance to it (e.g. The House in the Cerulean Sea, Avatar: The Last Airbender).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Bittersweet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real existential adversity (mortality, loss, the passage of time -- not politically "resistable") + connection/kindness deliberately chosen anyway, knowing it will cost grief later (e.g. Frieren).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not sufficient for any variant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simply having a hopeful tone or a happy ending. Most tier 1-4 works are correctly Hopepunk = No.</t>
   </si>
   <si>
     <t xml:space="preserve">Work</t>
@@ -2184,11 +2223,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="71486027"/>
-        <c:axId val="26757166"/>
+        <c:axId val="43826828"/>
+        <c:axId val="79257990"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="71486027"/>
+        <c:axId val="43826828"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2233,7 +2272,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26757166"/>
+        <c:crossAx val="79257990"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2241,7 +2280,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="26757166"/>
+        <c:axId val="79257990"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2286,7 +2325,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71486027"/>
+        <c:crossAx val="43826828"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2543,9 +2582,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>608400</xdr:colOff>
+      <xdr:colOff>608040</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>187560</xdr:rowOff>
+      <xdr:rowOff>187200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2554,7 +2593,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4889160" cy="3426120"/>
+        <a:ext cx="4888800" cy="3425760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2724,7 +2763,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
@@ -3094,6 +3133,59 @@
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>48</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3136,19 +3228,19 @@
         <v>25</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="H1" s="6" t="s">
         <v>7</v>
@@ -3172,16 +3264,16 @@
         <v>19</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3192,19 +3284,19 @@
         <v>26</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H2" s="8" t="n">
         <v>0.1</v>
@@ -3240,7 +3332,7 @@
         <v>1</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3251,19 +3343,19 @@
         <v>26</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H3" s="8" t="n">
         <v>0.2</v>
@@ -3299,7 +3391,7 @@
         <v>1</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3310,19 +3402,19 @@
         <v>26</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H4" s="8" t="n">
         <v>0.1</v>
@@ -3358,7 +3450,7 @@
         <v>1</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3369,19 +3461,19 @@
         <v>26</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H5" s="8" t="n">
         <v>0.1</v>
@@ -3417,7 +3509,7 @@
         <v>1</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3428,19 +3520,19 @@
         <v>27</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H6" s="8" t="n">
         <v>0.45</v>
@@ -3476,7 +3568,7 @@
         <v>2</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3487,19 +3579,19 @@
         <v>27</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="H7" s="8" t="n">
         <v>0.45</v>
@@ -3535,7 +3627,7 @@
         <v>2</v>
       </c>
       <c r="R7" s="3" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3546,19 +3638,19 @@
         <v>27</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H8" s="8" t="n">
         <v>0.45</v>
@@ -3594,7 +3686,7 @@
         <v>2</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3605,19 +3697,19 @@
         <v>27</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H9" s="8" t="n">
         <v>0.45</v>
@@ -3653,7 +3745,7 @@
         <v>2</v>
       </c>
       <c r="R9" s="3" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3664,19 +3756,19 @@
         <v>27</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H10" s="8" t="n">
         <v>0.45</v>
@@ -3712,7 +3804,7 @@
         <v>2</v>
       </c>
       <c r="R10" s="3" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3723,19 +3815,19 @@
         <v>27</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H11" s="8" t="n">
         <v>0.45</v>
@@ -3771,7 +3863,7 @@
         <v>2</v>
       </c>
       <c r="R11" s="3" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3782,19 +3874,19 @@
         <v>27</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H12" s="8" t="n">
         <v>0.45</v>
@@ -3830,7 +3922,7 @@
         <v>2</v>
       </c>
       <c r="R12" s="3" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3841,19 +3933,19 @@
         <v>27</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H13" s="8" t="n">
         <v>0.45</v>
@@ -3889,7 +3981,7 @@
         <v>2</v>
       </c>
       <c r="R13" s="3" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3900,19 +3992,19 @@
         <v>27</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H14" s="8" t="n">
         <v>0.45</v>
@@ -3948,7 +4040,7 @@
         <v>2</v>
       </c>
       <c r="R14" s="3" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3959,19 +4051,19 @@
         <v>27</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H15" s="8" t="n">
         <v>0.45</v>
@@ -4007,7 +4099,7 @@
         <v>2</v>
       </c>
       <c r="R15" s="3" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4018,19 +4110,19 @@
         <v>27</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H16" s="8" t="n">
         <v>0.45</v>
@@ -4066,7 +4158,7 @@
         <v>2</v>
       </c>
       <c r="R16" s="3" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4077,19 +4169,19 @@
         <v>27</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H17" s="8" t="n">
         <v>0.45</v>
@@ -4125,7 +4217,7 @@
         <v>2</v>
       </c>
       <c r="R17" s="3" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4136,19 +4228,19 @@
         <v>27</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H18" s="8" t="n">
         <v>0.45</v>
@@ -4184,7 +4276,7 @@
         <v>2</v>
       </c>
       <c r="R18" s="3" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4195,19 +4287,19 @@
         <v>28</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H19" s="8" t="n">
         <v>0.85</v>
@@ -4243,7 +4335,7 @@
         <v>3</v>
       </c>
       <c r="R19" s="3" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4254,19 +4346,19 @@
         <v>28</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H20" s="8" t="n">
         <v>0.85</v>
@@ -4302,7 +4394,7 @@
         <v>3</v>
       </c>
       <c r="R20" s="3" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4313,19 +4405,19 @@
         <v>28</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H21" s="8" t="n">
         <v>0.85</v>
@@ -4361,7 +4453,7 @@
         <v>3</v>
       </c>
       <c r="R21" s="3" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4372,19 +4464,19 @@
         <v>28</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H22" s="8" t="n">
         <v>0.85</v>
@@ -4420,7 +4512,7 @@
         <v>3</v>
       </c>
       <c r="R22" s="3" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4431,19 +4523,19 @@
         <v>28</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H23" s="8" t="n">
         <v>0.85</v>
@@ -4479,7 +4571,7 @@
         <v>3</v>
       </c>
       <c r="R23" s="3" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4490,19 +4582,19 @@
         <v>28</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H24" s="8" t="n">
         <v>0.85</v>
@@ -4538,7 +4630,7 @@
         <v>3</v>
       </c>
       <c r="R24" s="3" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4549,19 +4641,19 @@
         <v>28</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H25" s="8" t="n">
         <v>1.05</v>
@@ -4597,7 +4689,7 @@
         <v>3</v>
       </c>
       <c r="R25" s="3" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4608,19 +4700,19 @@
         <v>28</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H26" s="8" t="n">
         <v>1</v>
@@ -4656,7 +4748,7 @@
         <v>3</v>
       </c>
       <c r="R26" s="3" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4667,19 +4759,19 @@
         <v>28</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H27" s="8" t="n">
         <v>0.85</v>
@@ -4715,7 +4807,7 @@
         <v>3</v>
       </c>
       <c r="R27" s="3" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4726,19 +4818,19 @@
         <v>28</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H28" s="8" t="n">
         <v>1</v>
@@ -4774,7 +4866,7 @@
         <v>3</v>
       </c>
       <c r="R28" s="3" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4785,19 +4877,19 @@
         <v>28</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H29" s="8" t="n">
         <v>0.95</v>
@@ -4833,7 +4925,7 @@
         <v>3</v>
       </c>
       <c r="R29" s="3" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4844,19 +4936,19 @@
         <v>28</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H30" s="8" t="n">
         <v>0.85</v>
@@ -4892,7 +4984,7 @@
         <v>3</v>
       </c>
       <c r="R30" s="3" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4903,19 +4995,19 @@
         <v>28</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H31" s="8" t="n">
         <v>1</v>
@@ -4951,7 +5043,7 @@
         <v>3</v>
       </c>
       <c r="R31" s="3" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4962,19 +5054,19 @@
         <v>28</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H32" s="8" t="n">
         <v>0.95</v>
@@ -5010,7 +5102,7 @@
         <v>3</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5021,19 +5113,19 @@
         <v>28</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H33" s="8" t="n">
         <v>0.85</v>
@@ -5069,7 +5161,7 @@
         <v>3</v>
       </c>
       <c r="R33" s="3" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5080,19 +5172,19 @@
         <v>29</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H34" s="8" t="n">
         <v>1.25</v>
@@ -5128,7 +5220,7 @@
         <v>4</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5139,19 +5231,19 @@
         <v>29</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H35" s="8" t="n">
         <v>1.35</v>
@@ -5187,7 +5279,7 @@
         <v>4</v>
       </c>
       <c r="R35" s="3" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5198,19 +5290,19 @@
         <v>29</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H36" s="8" t="n">
         <v>1.35</v>
@@ -5246,7 +5338,7 @@
         <v>4</v>
       </c>
       <c r="R36" s="3" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5257,19 +5349,19 @@
         <v>29</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H37" s="8" t="n">
         <v>1.55</v>
@@ -5305,7 +5397,7 @@
         <v>4</v>
       </c>
       <c r="R37" s="3" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5316,19 +5408,19 @@
         <v>29</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H38" s="8" t="n">
         <v>1.25</v>
@@ -5364,7 +5456,7 @@
         <v>4</v>
       </c>
       <c r="R38" s="3" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5375,19 +5467,19 @@
         <v>29</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H39" s="8" t="n">
         <v>1.45</v>
@@ -5423,7 +5515,7 @@
         <v>4</v>
       </c>
       <c r="R39" s="3" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5434,19 +5526,19 @@
         <v>29</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H40" s="8" t="n">
         <v>1.25</v>
@@ -5482,7 +5574,7 @@
         <v>4</v>
       </c>
       <c r="R40" s="3" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5493,19 +5585,19 @@
         <v>29</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H41" s="8" t="n">
         <v>1.25</v>
@@ -5541,7 +5633,7 @@
         <v>4</v>
       </c>
       <c r="R41" s="3" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5552,19 +5644,19 @@
         <v>29</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H42" s="8" t="n">
         <v>1.4</v>
@@ -5600,7 +5692,7 @@
         <v>4</v>
       </c>
       <c r="R42" s="3" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5611,19 +5703,19 @@
         <v>29</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H43" s="8" t="n">
         <v>1.25</v>
@@ -5659,7 +5751,7 @@
         <v>4</v>
       </c>
       <c r="R43" s="3" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5670,19 +5762,19 @@
         <v>29</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H44" s="8" t="n">
         <v>1.25</v>
@@ -5718,7 +5810,7 @@
         <v>4</v>
       </c>
       <c r="R44" s="3" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5729,19 +5821,19 @@
         <v>29</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H45" s="8" t="n">
         <v>1.35</v>
@@ -5777,7 +5869,7 @@
         <v>4</v>
       </c>
       <c r="R45" s="3" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5788,19 +5880,19 @@
         <v>29</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H46" s="8" t="n">
         <v>1.25</v>
@@ -5836,7 +5928,7 @@
         <v>4</v>
       </c>
       <c r="R46" s="3" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5847,19 +5939,19 @@
         <v>29</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H47" s="8" t="n">
         <v>1.4</v>
@@ -5895,7 +5987,7 @@
         <v>4</v>
       </c>
       <c r="R47" s="3" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5906,19 +5998,19 @@
         <v>29</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H48" s="8" t="n">
         <v>1.25</v>
@@ -5954,7 +6046,7 @@
         <v>4</v>
       </c>
       <c r="R48" s="3" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5965,19 +6057,19 @@
         <v>29</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H49" s="8" t="n">
         <v>1.25</v>
@@ -6013,7 +6105,7 @@
         <v>4</v>
       </c>
       <c r="R49" s="3" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6024,19 +6116,19 @@
         <v>29</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H50" s="8" t="n">
         <v>1.25</v>
@@ -6072,7 +6164,7 @@
         <v>4</v>
       </c>
       <c r="R50" s="3" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6083,19 +6175,19 @@
         <v>29</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H51" s="8" t="n">
         <v>1.25</v>
@@ -6131,7 +6223,7 @@
         <v>4</v>
       </c>
       <c r="R51" s="3" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6142,19 +6234,19 @@
         <v>29</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H52" s="8" t="n">
         <v>1.4</v>
@@ -6190,7 +6282,7 @@
         <v>4</v>
       </c>
       <c r="R52" s="3" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6201,19 +6293,19 @@
         <v>29</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H53" s="8" t="n">
         <v>1.25</v>
@@ -6249,7 +6341,7 @@
         <v>4</v>
       </c>
       <c r="R53" s="3" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6260,19 +6352,19 @@
         <v>30</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H54" s="8" t="n">
         <v>1.85</v>
@@ -6308,7 +6400,7 @@
         <v>5</v>
       </c>
       <c r="R54" s="3" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6319,19 +6411,19 @@
         <v>30</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H55" s="8" t="n">
         <v>1.85</v>
@@ -6367,7 +6459,7 @@
         <v>5</v>
       </c>
       <c r="R55" s="3" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6378,19 +6470,19 @@
         <v>30</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H56" s="8" t="n">
         <v>2</v>
@@ -6426,7 +6518,7 @@
         <v>5</v>
       </c>
       <c r="R56" s="3" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6437,19 +6529,19 @@
         <v>30</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H57" s="8" t="n">
         <v>1.7</v>
@@ -6485,7 +6577,7 @@
         <v>5</v>
       </c>
       <c r="R57" s="3" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6496,19 +6588,19 @@
         <v>30</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H58" s="8" t="n">
         <v>1.9</v>
@@ -6544,7 +6636,7 @@
         <v>5</v>
       </c>
       <c r="R58" s="3" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6555,19 +6647,19 @@
         <v>30</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H59" s="8" t="n">
         <v>1.95</v>
@@ -6603,7 +6695,7 @@
         <v>5</v>
       </c>
       <c r="R59" s="3" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6614,19 +6706,19 @@
         <v>30</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H60" s="8" t="n">
         <v>1.95</v>
@@ -6662,7 +6754,7 @@
         <v>5</v>
       </c>
       <c r="R60" s="3" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6673,19 +6765,19 @@
         <v>30</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H61" s="8" t="n">
         <v>1.9</v>
@@ -6721,7 +6813,7 @@
         <v>5</v>
       </c>
       <c r="R61" s="3" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6732,19 +6824,19 @@
         <v>30</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H62" s="8" t="n">
         <v>1.7</v>
@@ -6780,7 +6872,7 @@
         <v>5</v>
       </c>
       <c r="R62" s="3" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6791,19 +6883,19 @@
         <v>31</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H63" s="8" t="n">
         <v>2.4</v>
@@ -6839,7 +6931,7 @@
         <v>6</v>
       </c>
       <c r="R63" s="3" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6850,19 +6942,19 @@
         <v>31</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H64" s="8" t="n">
         <v>2.2</v>
@@ -6898,7 +6990,7 @@
         <v>6</v>
       </c>
       <c r="R64" s="3" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6909,19 +7001,19 @@
         <v>31</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H65" s="8" t="n">
         <v>2.2</v>
@@ -6957,7 +7049,7 @@
         <v>6</v>
       </c>
       <c r="R65" s="3" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6968,19 +7060,19 @@
         <v>31</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H66" s="8" t="n">
         <v>2.35</v>
@@ -7016,7 +7108,7 @@
         <v>6</v>
       </c>
       <c r="R66" s="3" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7027,19 +7119,19 @@
         <v>31</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H67" s="8" t="n">
         <v>2.2</v>
@@ -7075,7 +7167,7 @@
         <v>6</v>
       </c>
       <c r="R67" s="3" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7086,19 +7178,19 @@
         <v>32</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H68" s="8" t="n">
         <v>2.95</v>
@@ -7134,7 +7226,7 @@
         <v>7</v>
       </c>
       <c r="R68" s="3" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7145,19 +7237,19 @@
         <v>33</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H69" s="8" t="n">
         <v>3.2</v>
@@ -7193,7 +7285,7 @@
         <v>8</v>
       </c>
       <c r="R69" s="3" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7204,19 +7296,19 @@
         <v>33</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H70" s="8" t="n">
         <v>3.5</v>
@@ -7252,7 +7344,7 @@
         <v>8</v>
       </c>
       <c r="R70" s="3" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7263,19 +7355,19 @@
         <v>33</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H71" s="8" t="n">
         <v>3.2</v>
@@ -7311,7 +7403,7 @@
         <v>8</v>
       </c>
       <c r="R71" s="3" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7322,19 +7414,19 @@
         <v>33</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H72" s="8" t="n">
         <v>3.2</v>
@@ -7370,7 +7462,7 @@
         <v>8</v>
       </c>
       <c r="R72" s="3" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7381,19 +7473,19 @@
         <v>34</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H73" s="8" t="n">
         <v>3.6</v>
@@ -7429,7 +7521,7 @@
         <v>9</v>
       </c>
       <c r="R73" s="3" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7440,19 +7532,19 @@
         <v>35</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H74" s="8" t="n">
         <v>4</v>
@@ -7488,7 +7580,7 @@
         <v>10</v>
       </c>
       <c r="R74" s="3" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7499,19 +7591,19 @@
         <v>27</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H75" s="1" t="n">
         <v>0.3</v>
@@ -7547,7 +7639,7 @@
         <v>2</v>
       </c>
       <c r="R75" s="1" t="s">
-        <v>267</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -7613,7 +7705,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -7629,10 +7721,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>270</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Sync tier category names to current site titles
Methodology, Summary, and Evaluations (Category column, 53 rows
across tiers 1-4) still had the pre-iteration tier names from before
all the title changes made directly on the live site. Tiers 5-10 were
already correct (never renamed). No effect on any score or formula --
Category is descriptive only.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -102,16 +102,16 @@
     <t xml:space="preserve">Category</t>
   </si>
   <si>
-    <t xml:space="preserve">Cozy Fantasy, Hopepunk &amp; Very Bright Fantasy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hopepunk, Cozy Fantasy &amp; Heroic Fantasy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Balanced, Melancholic or Hopepunk Fantasy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dark Fantasy with Hope</t>
+    <t xml:space="preserve">Wholesome Cozy Fantasy, Gentle Hopepunk &amp; Very Bright Fantasy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resilient Cozy Fantasy, Fierce Hopepunk &amp; Heroic Fantasy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantasy in Gray Tones</t>
   </si>
   <si>
     <t xml:space="preserve">Gloomy Fantasy</t>
@@ -2223,11 +2223,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="43826828"/>
-        <c:axId val="79257990"/>
+        <c:axId val="26245704"/>
+        <c:axId val="52466607"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="43826828"/>
+        <c:axId val="26245704"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2272,7 +2272,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79257990"/>
+        <c:crossAx val="52466607"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2280,7 +2280,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79257990"/>
+        <c:axId val="52466607"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2325,7 +2325,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43826828"/>
+        <c:crossAx val="26245704"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2582,9 +2582,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>608040</xdr:colOff>
+      <xdr:colOff>607680</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>187200</xdr:rowOff>
+      <xdr:rowOff>186840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2593,7 +2593,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4888800" cy="3425760"/>
+        <a:ext cx="4888440" cy="3425400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3134,7 +3134,7 @@
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>36</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>38</v>
       </c>
@@ -3150,12 +3150,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
         <v>41</v>
       </c>
@@ -3163,7 +3163,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
         <v>43</v>
       </c>
@@ -3171,7 +3171,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
         <v>45</v>
       </c>
@@ -3179,7 +3179,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
Add Adventure Time to tier 3 (score 2.68)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="288">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -865,6 +865,18 @@
   </si>
   <si>
     <t xml:space="preserve">A gentle, melancholic fable about loss, love, and learning to truly see — treated with poignant restraint rather than grimness.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adventure Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TV / Comics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendleton Ward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The post-Mushroom-War setting and Ice King's tragic loss of self add real melancholy, but whimsical humor and consistently effective heroism keep the tone gentle overall.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2194,7 +2206,7 @@
                   <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>20</c:v>
@@ -2223,11 +2235,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="26245704"/>
-        <c:axId val="52466607"/>
+        <c:axId val="10681028"/>
+        <c:axId val="15025122"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="26245704"/>
+        <c:axId val="10681028"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2272,7 +2284,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52466607"/>
+        <c:crossAx val="15025122"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2280,7 +2292,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52466607"/>
+        <c:axId val="15025122"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2325,7 +2337,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26245704"/>
+        <c:crossAx val="10681028"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2582,9 +2594,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>607680</xdr:colOff>
+      <xdr:colOff>607320</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>186840</xdr:rowOff>
+      <xdr:rowOff>186480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2593,7 +2605,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4888440" cy="3425400"/>
+        <a:ext cx="4888080" cy="3425040"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3206,7 +3218,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R75"/>
+  <dimension ref="A1:R76"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -7640,6 +7652,65 @@
       </c>
       <c r="R75" s="1" t="s">
         <v>280</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H76" s="1" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I76" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J76" s="1" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K76" s="1" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="L76" s="1" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="M76" s="1" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N76" s="1" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="O76" s="1" t="n">
+        <f aca="false">H76*Methodology!$E$4+I76*Methodology!$E$5+J76*Methodology!$E$6+K76*Methodology!$E$7+L76*Methodology!$E$8+M76*Methodology!$E$9+N76*Methodology!$E$10</f>
+        <v>0.745</v>
+      </c>
+      <c r="P76" s="1" t="n">
+        <f aca="false">1+(O76*2.25)</f>
+        <v>2.67625</v>
+      </c>
+      <c r="Q76" s="1" t="n">
+        <f aca="false">ROUND(P76,0)</f>
+        <v>3</v>
+      </c>
+      <c r="R76" s="1" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -7705,7 +7776,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -7721,10 +7792,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7768,11 +7839,11 @@
       </c>
       <c r="C6" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A6)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D6" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A6,Evaluations!$P$2:$P$200)</f>
-        <v>2.738125</v>
+        <v>2.7342578125</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Star vs. the Forces of Evil to tier 4 (score 3.75)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="291">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -877,6 +877,15 @@
   </si>
   <si>
     <t xml:space="preserve">The post-Mushroom-War setting and Ice King's tragic loss of self add real melancholy, but whimsical humor and consistently effective heroism keep the tone gentle overall.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Star vs. the Forces of Evil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daron Nefcy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generations of Mewman genocide against Monsters drive the later seasons, and the finale resolves the conflict by erasing magic outright rather than reforming the system — heavier than most gray-tones peers, though Star's reconciliation arc and the show's comedic early seasons keep real hope in the frame.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2209,7 +2218,7 @@
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>9</c:v>
@@ -2235,11 +2244,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="10681028"/>
-        <c:axId val="15025122"/>
+        <c:axId val="73284355"/>
+        <c:axId val="81184856"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="10681028"/>
+        <c:axId val="73284355"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2284,7 +2293,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15025122"/>
+        <c:crossAx val="81184856"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2292,7 +2301,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="15025122"/>
+        <c:axId val="81184856"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2337,7 +2346,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10681028"/>
+        <c:crossAx val="73284355"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2594,9 +2603,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>607320</xdr:colOff>
+      <xdr:colOff>606960</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>186480</xdr:rowOff>
+      <xdr:rowOff>186120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2605,7 +2614,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4888080" cy="3425040"/>
+        <a:ext cx="4887720" cy="3424680"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3218,7 +3227,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R76"/>
+  <dimension ref="A1:R77"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -7654,7 +7663,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="n">
         <v>3</v>
       </c>
@@ -7711,6 +7720,65 @@
       </c>
       <c r="R76" s="1" t="s">
         <v>284</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H77" s="1" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I77" s="1" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J77" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K77" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L77" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M77" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="N77" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="O77" s="1" t="n">
+        <f aca="false">H77*Methodology!$E$4+I77*Methodology!$E$5+J77*Methodology!$E$6+K77*Methodology!$E$7+L77*Methodology!$E$8+M77*Methodology!$E$9+N77*Methodology!$E$10</f>
+        <v>1.2225</v>
+      </c>
+      <c r="P77" s="1" t="n">
+        <f aca="false">1+(O77*2.25)</f>
+        <v>3.750625</v>
+      </c>
+      <c r="Q77" s="1" t="n">
+        <f aca="false">ROUND(P77,0)</f>
+        <v>4</v>
+      </c>
+      <c r="R77" s="1" t="s">
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -7776,7 +7844,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -7792,10 +7860,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7855,11 +7923,11 @@
       </c>
       <c r="C7" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A7)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A7,Evaluations!$P$2:$P$200)</f>
-        <v>3.77340625</v>
+        <v>3.77232142857143</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Clevatess to tier 6 (score 5.85)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="294">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -886,6 +886,15 @@
   </si>
   <si>
     <t xml:space="preserve">Generations of Mewman genocide against Monsters drive the later seasons, and the finale resolves the conflict by erasing magic outright rather than reforming the system — heavier than most gray-tones peers, though Star's reconciliation arc and the show's comedic early seasons keep real hope in the frame.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clevatess</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yūji Iwahara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A demon king raising a human infant instead of annihilating humanity is genuinely tender, but the surrounding world is severe — infant trafficking and experimentation, and a named character's backstory of sustained abuse push explicit darkness above most of this tier.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2224,7 +2233,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>1</c:v>
@@ -2244,11 +2253,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="73284355"/>
-        <c:axId val="81184856"/>
+        <c:axId val="79935928"/>
+        <c:axId val="93522527"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="73284355"/>
+        <c:axId val="79935928"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2293,7 +2302,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81184856"/>
+        <c:crossAx val="93522527"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2301,7 +2310,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="81184856"/>
+        <c:axId val="93522527"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2346,7 +2355,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73284355"/>
+        <c:crossAx val="79935928"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2603,9 +2612,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>606960</xdr:colOff>
+      <xdr:colOff>606600</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>186120</xdr:rowOff>
+      <xdr:rowOff>185760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2614,7 +2623,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4887720" cy="3424680"/>
+        <a:ext cx="4887360" cy="3424320"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3227,7 +3236,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R77"/>
+  <dimension ref="A1:R78"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -7722,7 +7731,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="n">
         <v>4</v>
       </c>
@@ -7779,6 +7788,65 @@
       </c>
       <c r="R77" s="1" t="s">
         <v>287</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H78" s="1" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="I78" s="1" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J78" s="1" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K78" s="1" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="L78" s="1" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="M78" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N78" s="1" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="O78" s="1" t="n">
+        <f aca="false">H78*Methodology!$E$4+I78*Methodology!$E$5+J78*Methodology!$E$6+K78*Methodology!$E$7+L78*Methodology!$E$8+M78*Methodology!$E$9+N78*Methodology!$E$10</f>
+        <v>2.155</v>
+      </c>
+      <c r="P78" s="1" t="n">
+        <f aca="false">1+(O78*2.25)</f>
+        <v>5.84875</v>
+      </c>
+      <c r="Q78" s="1" t="n">
+        <f aca="false">ROUND(P78,0)</f>
+        <v>6</v>
+      </c>
+      <c r="R78" s="1" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -7844,7 +7912,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -7860,10 +7928,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7955,11 +8023,11 @@
       </c>
       <c r="C9" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A9)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A9,Evaluations!$P$2:$P$200)</f>
-        <v>6.0445</v>
+        <v>6.011875</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add The Saga of Tanya the Evil to tier 7 (score 7.30)
Tier 7 now has two works, so its layout switches from the single-item
"solo" centered style to the standard multi-column grid.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="298">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -895,6 +895,18 @@
   </si>
   <si>
     <t xml:space="preserve">A demon king raising a human infant instead of annihilating humanity is genuinely tender, but the surrounding world is severe — infant trafficking and experimentation, and a named character's backstory of sustained abuse push explicit darkness above most of this tier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Saga of Tanya the Evil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Light Novels / Manga / Anime / Film</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carlo Zen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A reincarnated corporate pragmatist becomes a ruthlessly effective officer in a magic-augmented World War I that never ends; the satire's thesis is that cynicism outperforms idealism, and neither Tanya nor the war itself ever really changes.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2236,7 +2248,7 @@
                   <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>4</c:v>
@@ -2253,11 +2265,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="79935928"/>
-        <c:axId val="93522527"/>
+        <c:axId val="80746475"/>
+        <c:axId val="19812678"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="79935928"/>
+        <c:axId val="80746475"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2302,7 +2314,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93522527"/>
+        <c:crossAx val="19812678"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2310,7 +2322,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93522527"/>
+        <c:axId val="19812678"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2355,7 +2367,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79935928"/>
+        <c:crossAx val="80746475"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2612,9 +2624,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>606600</xdr:colOff>
+      <xdr:colOff>606240</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>185760</xdr:rowOff>
+      <xdr:rowOff>185400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2623,7 +2635,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4887360" cy="3424320"/>
+        <a:ext cx="4887000" cy="3423960"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3236,7 +3248,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R78"/>
+  <dimension ref="A1:R79"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -7790,7 +7802,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="n">
         <v>6</v>
       </c>
@@ -7847,6 +7859,65 @@
       </c>
       <c r="R78" s="1" t="s">
         <v>290</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H79" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I79" s="1" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J79" s="1" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="K79" s="1" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="L79" s="1" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M79" s="1" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="N79" s="1" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="O79" s="1" t="n">
+        <f aca="false">H79*Methodology!$E$4+I79*Methodology!$E$5+J79*Methodology!$E$6+K79*Methodology!$E$7+L79*Methodology!$E$8+M79*Methodology!$E$9+N79*Methodology!$E$10</f>
+        <v>2.8</v>
+      </c>
+      <c r="P79" s="1" t="n">
+        <f aca="false">1+(O79*2.25)</f>
+        <v>7.3</v>
+      </c>
+      <c r="Q79" s="1" t="n">
+        <f aca="false">ROUND(P79,0)</f>
+        <v>7</v>
+      </c>
+      <c r="R79" s="1" t="s">
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -7912,7 +7983,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -7928,10 +7999,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8039,11 +8110,11 @@
       </c>
       <c r="C10" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A10)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A10,Evaluations!$P$2:$P$200)</f>
-        <v>7.31125</v>
+        <v>7.305625</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Re:Zero - Starting Life in Another World to tier 6 (score 5.82)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="301">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -907,6 +907,15 @@
   </si>
   <si>
     <t xml:space="preserve">A reincarnated corporate pragmatist becomes a ruthlessly effective officer in a magic-augmented World War I that never ends; the satire's thesis is that cynicism outperforms idealism, and neither Tanya nor the war itself ever really changes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re:Zero − Starting Life in Another World</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tappei Nagatsuki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subaru's “Return by Death” turns failure into genuinely repeated, graphic trauma — among the most psychologically brutal content on this scale — but the loops consistently let heroism and hard-won found-family actually fix things, so it stays a story about earning growth through suffering rather than accepting defeat.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2245,7 +2254,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>2</c:v>
@@ -2265,11 +2274,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="80746475"/>
-        <c:axId val="19812678"/>
+        <c:axId val="9167800"/>
+        <c:axId val="31666420"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="80746475"/>
+        <c:axId val="9167800"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2314,7 +2323,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19812678"/>
+        <c:crossAx val="31666420"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2322,7 +2331,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19812678"/>
+        <c:axId val="31666420"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2367,7 +2376,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80746475"/>
+        <c:crossAx val="9167800"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2624,9 +2633,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>606240</xdr:colOff>
+      <xdr:colOff>605880</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>185400</xdr:rowOff>
+      <xdr:rowOff>185040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2635,7 +2644,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4887000" cy="3423960"/>
+        <a:ext cx="4886640" cy="3423600"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3248,7 +3257,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R79"/>
+  <dimension ref="A1:R80"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -7861,7 +7870,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="n">
         <v>7</v>
       </c>
@@ -7918,6 +7927,65 @@
       </c>
       <c r="R79" s="1" t="s">
         <v>294</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H80" s="1" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="I80" s="1" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J80" s="1" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="K80" s="1" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="L80" s="1" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M80" s="1" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="N80" s="1" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="O80" s="1" t="n">
+        <f aca="false">H80*Methodology!$E$4+I80*Methodology!$E$5+J80*Methodology!$E$6+K80*Methodology!$E$7+L80*Methodology!$E$8+M80*Methodology!$E$9+N80*Methodology!$E$10</f>
+        <v>2.14</v>
+      </c>
+      <c r="P80" s="1" t="n">
+        <f aca="false">1+(O80*2.25)</f>
+        <v>5.815</v>
+      </c>
+      <c r="Q80" s="1" t="n">
+        <f aca="false">ROUND(P80,0)</f>
+        <v>6</v>
+      </c>
+      <c r="R80" s="1" t="s">
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -7983,7 +8051,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -7999,10 +8067,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8094,11 +8162,11 @@
       </c>
       <c r="C9" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A9)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D9" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A9,Evaluations!$P$2:$P$200)</f>
-        <v>6.011875</v>
+        <v>5.98375</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Rename tier 7/8 categories: split the Grimdark cluster
Tier 6 (Dark Fantasy) and tier 7 now form a matched pair, with tier 7
becoming Extreme Dark Fantasy / Fantasía oscura extrema instead of a
third "Grimdark" variant. Tier 8 simplifies to plain Grimdark, which
then intensifies cleanly into tier 9 (Extreme Grimdark) and tier 10
(Very Extreme Grimdark). Updated in index.html, es/index.html, and the
xlsx (Methodology tier list, Evaluations Category column for the
affected rows, Summary sheet).
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -120,10 +120,10 @@
     <t xml:space="preserve">Dark Fantasy</t>
   </si>
   <si>
+    <t xml:space="preserve">Extreme Dark Fantasy</t>
+  </si>
+  <si>
     <t xml:space="preserve">Grimdark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Intense Grimdark</t>
   </si>
   <si>
     <t xml:space="preserve">Extreme Grimdark</t>
@@ -2274,11 +2274,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="9167800"/>
-        <c:axId val="31666420"/>
+        <c:axId val="49869824"/>
+        <c:axId val="88565798"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="9167800"/>
+        <c:axId val="49869824"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2323,7 +2323,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31666420"/>
+        <c:crossAx val="88565798"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2331,7 +2331,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="31666420"/>
+        <c:axId val="88565798"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2376,7 +2376,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9167800"/>
+        <c:crossAx val="49869824"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2633,9 +2633,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>605880</xdr:colOff>
+      <xdr:colOff>605520</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>185040</xdr:rowOff>
+      <xdr:rowOff>184680</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2644,7 +2644,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4886640" cy="3423600"/>
+        <a:ext cx="4886280" cy="3423240"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -7929,7 +7929,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="n">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
Add Legend (1985) to tier 2 (score 1.91)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="304">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -916,6 +916,15 @@
   </si>
   <si>
     <t xml:space="preserve">Subaru's “Return by Death” turns failure into genuinely repeated, graphic trauma — among the most psychologically brutal content on this scale — but the loops consistently let heroism and hard-won found-family actually fix things, so it stays a story about earning growth through suffering rather than accepting defeat.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ridley Scott</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A mythic, single-villain fairy tale rather than anything institutional: Darkness's gothic menace and the stallion unicorn's death carry real atmospheric horror, but heroism is straightforward and decisive, and Lili's temptation is treated as innocence exploited rather than culpability.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2242,7 +2251,7 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>14</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>16</c:v>
@@ -2274,11 +2283,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="49869824"/>
-        <c:axId val="88565798"/>
+        <c:axId val="17943322"/>
+        <c:axId val="22242778"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="49869824"/>
+        <c:axId val="17943322"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2323,7 +2332,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88565798"/>
+        <c:crossAx val="22242778"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2331,7 +2340,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="88565798"/>
+        <c:axId val="22242778"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2376,7 +2385,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49869824"/>
+        <c:crossAx val="17943322"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2633,9 +2642,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>605520</xdr:colOff>
+      <xdr:colOff>605160</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>184680</xdr:rowOff>
+      <xdr:rowOff>184320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2644,7 +2653,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4886280" cy="3423240"/>
+        <a:ext cx="4885920" cy="3422880"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3257,7 +3266,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R80"/>
+  <dimension ref="A1:R81"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -7986,6 +7995,65 @@
       </c>
       <c r="R80" s="1" t="s">
         <v>297</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H81" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I81" s="1" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J81" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K81" s="1" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L81" s="1" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M81" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="N81" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="O81" s="1" t="n">
+        <f aca="false">H81*Methodology!$E$4+I81*Methodology!$E$5+J81*Methodology!$E$6+K81*Methodology!$E$7+L81*Methodology!$E$8+M81*Methodology!$E$9+N81*Methodology!$E$10</f>
+        <v>0.405</v>
+      </c>
+      <c r="P81" s="1" t="n">
+        <f aca="false">1+(O81*2.25)</f>
+        <v>1.91125</v>
+      </c>
+      <c r="Q81" s="1" t="n">
+        <f aca="false">ROUND(P81,0)</f>
+        <v>2</v>
+      </c>
+      <c r="R81" s="1" t="s">
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -8051,7 +8119,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -8067,10 +8135,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8098,11 +8166,11 @@
       </c>
       <c r="C5" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A5)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A5,Evaluations!$P$2:$P$200)</f>
-        <v>1.85339285714286</v>
+        <v>1.85725</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add The NeverEnding Story to tier 2 (score 2.11)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="307">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -925,6 +925,15 @@
   </si>
   <si>
     <t xml:space="preserve">A mythic, single-villain fairy tale rather than anything institutional: Darkness's gothic menace and the stallion unicorn's death carry real atmospheric horror, but heroism is straightforward and decisive, and Lili's temptation is treated as innocence exploited rather than culpability.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The NeverEnding Story</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michael Ende</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scored against the full novel, not just the 1984 film (which only adapts the first half): Artax's death and the Nothing's nihilism are real, but the book's second half — Bastian's own descent into cruelty once granted unlimited wish-power, and the hard-won cost of finding his way back to himself — adds real moral cynicism and redemption difficulty the film omits entirely.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2251,7 +2260,7 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>15</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>16</c:v>
@@ -2283,11 +2292,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="17943322"/>
-        <c:axId val="22242778"/>
+        <c:axId val="25202197"/>
+        <c:axId val="61689998"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="17943322"/>
+        <c:axId val="25202197"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2332,7 +2341,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22242778"/>
+        <c:crossAx val="61689998"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2340,7 +2349,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22242778"/>
+        <c:axId val="61689998"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2385,7 +2394,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17943322"/>
+        <c:crossAx val="25202197"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2642,9 +2651,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>605160</xdr:colOff>
+      <xdr:colOff>604800</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>184320</xdr:rowOff>
+      <xdr:rowOff>183960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2653,7 +2662,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4885920" cy="3422880"/>
+        <a:ext cx="4885560" cy="3422520"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3266,7 +3275,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R81"/>
+  <dimension ref="A1:R82"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -7997,7 +8006,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="n">
         <v>2</v>
       </c>
@@ -8054,6 +8063,65 @@
       </c>
       <c r="R81" s="1" t="s">
         <v>300</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H82" s="1" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I82" s="1" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J82" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K82" s="1" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L82" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M82" s="1" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N82" s="1" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="O82" s="1" t="n">
+        <f aca="false">H82*Methodology!$E$4+I82*Methodology!$E$5+J82*Methodology!$E$6+K82*Methodology!$E$7+L82*Methodology!$E$8+M82*Methodology!$E$9+N82*Methodology!$E$10</f>
+        <v>0.4925</v>
+      </c>
+      <c r="P82" s="1" t="n">
+        <f aca="false">1+(O82*2.25)</f>
+        <v>2.108125</v>
+      </c>
+      <c r="Q82" s="1" t="n">
+        <f aca="false">ROUND(P82,0)</f>
+        <v>2</v>
+      </c>
+      <c r="R82" s="1" t="s">
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -8119,7 +8187,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -8135,10 +8203,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8166,11 +8234,11 @@
       </c>
       <c r="C5" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A5)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A5,Evaluations!$P$2:$P$200)</f>
-        <v>1.85725</v>
+        <v>1.8729296875</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Shin Sekai Yori (From the New World) to tier 8 (score 8.41)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="311">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -934,6 +934,18 @@
   </si>
   <si>
     <t xml:space="preserve">Scored against the full novel, not just the 1984 film (which only adapts the first half): Artax's death and the Nothing's nihilism are real, but the book's second half — Bastian's own descent into cruelty once granted unlimited wish-power, and the hard-won cost of finding his way back to himself — adds real moral cynicism and redemption difficulty the film omits entirely.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shin Sekai Yori (From the New World)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novel / Anime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yusuke Kishi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A seemingly idyllic future society is built on secret child eugenics (killing children flagged as psychologically “unstable”) and the enslavement/extermination of the Queerats, who turn out to be humanity's own left-behind kin; the protagonists win a tactical victory but explicitly fail to dismantle the totalitarian system, which persists unchanged at the end.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2278,7 +2290,7 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>1</c:v>
@@ -2292,11 +2304,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="25202197"/>
-        <c:axId val="61689998"/>
+        <c:axId val="83786658"/>
+        <c:axId val="11467498"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="25202197"/>
+        <c:axId val="83786658"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2341,7 +2353,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61689998"/>
+        <c:crossAx val="11467498"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2349,7 +2361,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61689998"/>
+        <c:axId val="11467498"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2394,7 +2406,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25202197"/>
+        <c:crossAx val="83786658"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2651,9 +2663,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>604800</xdr:colOff>
+      <xdr:colOff>604440</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>183960</xdr:rowOff>
+      <xdr:rowOff>183600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2662,7 +2674,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4885560" cy="3422520"/>
+        <a:ext cx="4885200" cy="3422160"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3275,7 +3287,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R82"/>
+  <dimension ref="A1:R83"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -8065,7 +8077,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="n">
         <v>2</v>
       </c>
@@ -8122,6 +8134,65 @@
       </c>
       <c r="R82" s="1" t="s">
         <v>303</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H83" s="1" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="I83" s="1" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="J83" s="1" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="K83" s="1" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L83" s="1" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M83" s="1" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="N83" s="1" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="O83" s="1" t="n">
+        <f aca="false">H83*Methodology!$E$4+I83*Methodology!$E$5+J83*Methodology!$E$6+K83*Methodology!$E$7+L83*Methodology!$E$8+M83*Methodology!$E$9+N83*Methodology!$E$10</f>
+        <v>3.295</v>
+      </c>
+      <c r="P83" s="1" t="n">
+        <f aca="false">1+(O83*2.25)</f>
+        <v>8.41375</v>
+      </c>
+      <c r="Q83" s="1" t="n">
+        <f aca="false">ROUND(P83,0)</f>
+        <v>8</v>
+      </c>
+      <c r="R83" s="1" t="s">
+        <v>307</v>
       </c>
     </row>
   </sheetData>
@@ -8187,7 +8258,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -8203,10 +8274,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8330,11 +8401,11 @@
       </c>
       <c r="C11" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A11)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D11" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A11,Evaluations!$P$2:$P$200)</f>
-        <v>8.37859375</v>
+        <v>8.385625</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Mushishi to tier 2 (score 2.05)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="314">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -946,6 +946,15 @@
   </si>
   <si>
     <t xml:space="preserve">A seemingly idyllic future society is built on secret child eugenics (killing children flagged as psychologically “unstable”) and the enslavement/extermination of the Queerats, who turn out to be humanity's own left-behind kin; the protagonists win a tactical victory but explicitly fail to dismantle the totalitarian system, which persists unchanged at the end.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mushishi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yuki Urushibara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An anthology of quiet, often irreversible personal tragedy (permanent loss of a limb, a mother's death, lasting grief) rather than institutional darkness — there's no villain, no war, no system to critique, just impermanence met with care. Bittersweet Hopepunk: arguably the purest fit on this scale, since mortality-and-connection-anyway is the show's entire structure, not a framing device.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2272,7 +2281,7 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>16</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>16</c:v>
@@ -2304,11 +2313,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="83786658"/>
-        <c:axId val="11467498"/>
+        <c:axId val="74498014"/>
+        <c:axId val="21620591"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="83786658"/>
+        <c:axId val="74498014"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2353,7 +2362,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11467498"/>
+        <c:crossAx val="21620591"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2361,7 +2370,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11467498"/>
+        <c:axId val="21620591"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2406,7 +2415,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83786658"/>
+        <c:crossAx val="74498014"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2663,9 +2672,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>604440</xdr:colOff>
+      <xdr:colOff>604080</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>183600</xdr:rowOff>
+      <xdr:rowOff>183240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2674,7 +2683,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4885200" cy="3422160"/>
+        <a:ext cx="4884840" cy="3421800"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3287,7 +3296,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R83"/>
+  <dimension ref="A1:R84"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -8136,7 +8145,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="n">
         <v>8</v>
       </c>
@@ -8193,6 +8202,65 @@
       </c>
       <c r="R83" s="1" t="s">
         <v>307</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H84" s="1" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I84" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J84" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K84" s="1" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L84" s="1" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M84" s="1" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N84" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O84" s="1" t="n">
+        <f aca="false">H84*Methodology!$E$4+I84*Methodology!$E$5+J84*Methodology!$E$6+K84*Methodology!$E$7+L84*Methodology!$E$8+M84*Methodology!$E$9+N84*Methodology!$E$10</f>
+        <v>0.4675</v>
+      </c>
+      <c r="P84" s="1" t="n">
+        <f aca="false">1+(O84*2.25)</f>
+        <v>2.051875</v>
+      </c>
+      <c r="Q84" s="1" t="n">
+        <f aca="false">ROUND(P84,0)</f>
+        <v>2</v>
+      </c>
+      <c r="R84" s="1" t="s">
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -8258,7 +8326,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -8274,10 +8342,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8305,11 +8373,11 @@
       </c>
       <c r="C5" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A5)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A5,Evaluations!$P$2:$P$200)</f>
-        <v>1.8729296875</v>
+        <v>1.88345588235294</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Record of Lodoss War to tier 3 (score 2.74)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="318">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -955,6 +955,18 @@
   </si>
   <si>
     <t xml:space="preserve">An anthology of quiet, often irreversible personal tragedy (permanent loss of a limb, a mother's death, lasting grief) rather than institutional darkness — there's no villain, no war, no system to critique, just impermanence met with care. Bittersweet Hopepunk: arguably the purest fit on this scale, since mortality-and-connection-anyway is the show's entire structure, not a framing device.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Record of Lodoss War</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novels / Anime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ryo Mizuno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classic D&amp;D-inspired epic fantasy: the Marmo invasion costs both warring kings their lives and the party its dwarf, Ghim, in the finale, and the Grey Witch Karla's whole modus operandi is centuries of orchestrating wars to keep any nation from growing too powerful — but the heroes still win a decisive, restorative victory, keeping it in Dragonlance's company rather than heavier territory.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2284,7 +2296,7 @@
                   <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>21</c:v>
@@ -2313,11 +2325,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="74498014"/>
-        <c:axId val="21620591"/>
+        <c:axId val="54109588"/>
+        <c:axId val="55952649"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="74498014"/>
+        <c:axId val="54109588"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2362,7 +2374,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21620591"/>
+        <c:crossAx val="55952649"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2370,7 +2382,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="21620591"/>
+        <c:axId val="55952649"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2415,7 +2427,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74498014"/>
+        <c:crossAx val="54109588"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2672,9 +2684,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>604080</xdr:colOff>
+      <xdr:colOff>603720</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>183240</xdr:rowOff>
+      <xdr:rowOff>182880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2683,7 +2695,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4884840" cy="3421800"/>
+        <a:ext cx="4884480" cy="3421440"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3296,7 +3308,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R84"/>
+  <dimension ref="A1:R85"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -8204,7 +8216,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="n">
         <v>2</v>
       </c>
@@ -8261,6 +8273,65 @@
       </c>
       <c r="R84" s="1" t="s">
         <v>310</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H85" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I85" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J85" s="1" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K85" s="1" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="L85" s="1" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M85" s="1" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N85" s="1" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="O85" s="1" t="n">
+        <f aca="false">H85*Methodology!$E$4+I85*Methodology!$E$5+J85*Methodology!$E$6+K85*Methodology!$E$7+L85*Methodology!$E$8+M85*Methodology!$E$9+N85*Methodology!$E$10</f>
+        <v>0.775</v>
+      </c>
+      <c r="P85" s="1" t="n">
+        <f aca="false">1+(O85*2.25)</f>
+        <v>2.74375</v>
+      </c>
+      <c r="Q85" s="1" t="n">
+        <f aca="false">ROUND(P85,0)</f>
+        <v>3</v>
+      </c>
+      <c r="R85" s="1" t="s">
+        <v>314</v>
       </c>
     </row>
   </sheetData>
@@ -8326,7 +8397,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -8342,10 +8413,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8389,11 +8460,11 @@
       </c>
       <c r="C6" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A6)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A6,Evaluations!$P$2:$P$200)</f>
-        <v>2.7342578125</v>
+        <v>2.73481617647059</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add The Legend of Vox Machina to tier 4 (score 3.75)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="322">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -967,6 +967,18 @@
   </si>
   <si>
     <t xml:space="preserve">Classic D&amp;D-inspired epic fantasy: the Marmo invasion costs both warring kings their lives and the party its dwarf, Ghim, in the finale, and the Grey Witch Karla's whole modus operandi is centuries of orchestrating wars to keep any nation from growing too powerful — but the heroes still win a decisive, restorative victory, keeping it in Dragonlance's company rather than heavier territory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Legend of Vox Machina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical Role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TV-MA adult animation with real gore, a torture scene and on-screen child deaths, plus Percy's demon-fueled revenge arc and Vax'ildan's permanent death paying his soul to the Raven Queen — but the found-family heart, crude comedy, and consistently successful heroism (Whitestone liberated, Percy's darkness overcome) keep hope structurally dominant.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2299,7 +2311,7 @@
                   <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>21</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>9</c:v>
@@ -2325,11 +2337,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="54109588"/>
-        <c:axId val="55952649"/>
+        <c:axId val="72794581"/>
+        <c:axId val="93301847"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="54109588"/>
+        <c:axId val="72794581"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2374,7 +2386,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55952649"/>
+        <c:crossAx val="93301847"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2382,7 +2394,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55952649"/>
+        <c:axId val="93301847"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2427,7 +2439,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54109588"/>
+        <c:crossAx val="72794581"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2684,9 +2696,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>603720</xdr:colOff>
+      <xdr:colOff>603360</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>182880</xdr:rowOff>
+      <xdr:rowOff>182520</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2695,7 +2707,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4884480" cy="3421440"/>
+        <a:ext cx="4884120" cy="3421080"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3308,7 +3320,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R85"/>
+  <dimension ref="A1:R86"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -8275,7 +8287,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="n">
         <v>3</v>
       </c>
@@ -8332,6 +8344,65 @@
       </c>
       <c r="R85" s="1" t="s">
         <v>314</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H86" s="1" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I86" s="1" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J86" s="1" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="K86" s="1" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L86" s="1" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M86" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N86" s="1" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="O86" s="1" t="n">
+        <f aca="false">H86*Methodology!$E$4+I86*Methodology!$E$5+J86*Methodology!$E$6+K86*Methodology!$E$7+L86*Methodology!$E$8+M86*Methodology!$E$9+N86*Methodology!$E$10</f>
+        <v>1.22</v>
+      </c>
+      <c r="P86" s="1" t="n">
+        <f aca="false">1+(O86*2.25)</f>
+        <v>3.745</v>
+      </c>
+      <c r="Q86" s="1" t="n">
+        <f aca="false">ROUND(P86,0)</f>
+        <v>4</v>
+      </c>
+      <c r="R86" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
   </sheetData>
@@ -8397,7 +8468,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -8413,10 +8484,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8476,11 +8547,11 @@
       </c>
       <c r="C7" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A7)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A7,Evaluations!$P$2:$P$200)</f>
-        <v>3.77232142857143</v>
+        <v>3.77107954545455</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add The Nightmare Before Christmas to tier 1 (score 1.46)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="325">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -979,6 +979,15 @@
   </si>
   <si>
     <t xml:space="preserve">TV-MA adult animation with real gore, a torture scene and on-screen child deaths, plus Percy's demon-fueled revenge arc and Vax'ildan's permanent death paying his soul to the Raven Queen — but the found-family heart, crude comedy, and consistently successful heroism (Whitestone liberated, Percy's darkness overcome) keep hope structurally dominant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Nightmare Before Christmas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tim Burton / Henry Selick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gothic cotton candy: Oogie Boogie's sadistic gambling with Santa's life gives it real (if comedic) villain menace the gentlest Ghibli films don't have, but the whimsical Halloween Town community is fundamentally kind, Jack's mistake is quickly and fully undone, and the ending restores everything with romance blooming.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2302,7 +2311,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>17</c:v>
@@ -2337,11 +2346,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="72794581"/>
-        <c:axId val="93301847"/>
+        <c:axId val="27111044"/>
+        <c:axId val="81977665"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="72794581"/>
+        <c:axId val="27111044"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2386,7 +2395,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93301847"/>
+        <c:crossAx val="81977665"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2394,7 +2403,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93301847"/>
+        <c:axId val="81977665"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2439,7 +2448,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72794581"/>
+        <c:crossAx val="27111044"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2696,9 +2705,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>603360</xdr:colOff>
+      <xdr:colOff>603000</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>182520</xdr:rowOff>
+      <xdr:rowOff>182160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2707,7 +2716,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4884120" cy="3421080"/>
+        <a:ext cx="4883760" cy="3420720"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3320,7 +3329,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R86"/>
+  <dimension ref="A1:R87"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -8346,7 +8355,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="n">
         <v>4</v>
       </c>
@@ -8403,6 +8412,65 @@
       </c>
       <c r="R86" s="1" t="s">
         <v>318</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H87" s="1" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I87" s="1" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J87" s="1" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K87" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L87" s="1" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M87" s="1" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N87" s="1" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="O87" s="1" t="n">
+        <f aca="false">H87*Methodology!$E$4+I87*Methodology!$E$5+J87*Methodology!$E$6+K87*Methodology!$E$7+L87*Methodology!$E$8+M87*Methodology!$E$9+N87*Methodology!$E$10</f>
+        <v>0.205</v>
+      </c>
+      <c r="P87" s="1" t="n">
+        <f aca="false">1+(O87*2.25)</f>
+        <v>1.46125</v>
+      </c>
+      <c r="Q87" s="1" t="n">
+        <f aca="false">ROUND(P87,0)</f>
+        <v>1</v>
+      </c>
+      <c r="R87" s="1" t="s">
+        <v>321</v>
       </c>
     </row>
   </sheetData>
@@ -8468,7 +8536,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -8484,10 +8552,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8499,11 +8567,11 @@
       </c>
       <c r="C4" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A4)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A4,Evaluations!$P$2:$P$200)</f>
-        <v>1.15890625</v>
+        <v>1.219375</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Correct The Nightmare Before Christmas: move tier 1 -> tier 2 (1.46 -> 1.71)
The first pass underweighted Explicit Darkness relative to how much of
the film is spent in genuinely macabre horror-imagery (skeleton/monster
designs throughout, Sally's repeated self-dismemberment, Oogie Boogie
gambling with Santa's life) despite the plot resolving safely. Flagged
by the user as an inconsistency with tier 1's "Very Bright Fantasy"
register.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -987,7 +987,7 @@
     <t xml:space="preserve">Tim Burton / Henry Selick</t>
   </si>
   <si>
-    <t xml:space="preserve">Gothic cotton candy: Oogie Boogie's sadistic gambling with Santa's life gives it real (if comedic) villain menace the gentlest Ghibli films don't have, but the whimsical Halloween Town community is fundamentally kind, Jack's mistake is quickly and fully undone, and the ending restores everything with romance blooming.</t>
+    <t xml:space="preserve">Corrected from an earlier tier-1 placement: the pervasive Halloween Town horror aesthetic (skeleton/monster designs throughout, Sally's repeated self-dismemberment, Oogie Boogie sadistically gambling with Santa's life, children traumatized by monstrous gifts) is a lot of visible, disturbing content for a film whose plot ultimately resolves safely — Explicit Darkness was underweighted the first time.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2311,10 +2311,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>5</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>17</c:v>
@@ -2346,11 +2346,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="27111044"/>
-        <c:axId val="81977665"/>
+        <c:axId val="39755150"/>
+        <c:axId val="83895924"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="27111044"/>
+        <c:axId val="39755150"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2395,7 +2395,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81977665"/>
+        <c:crossAx val="83895924"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2403,7 +2403,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="81977665"/>
+        <c:axId val="83895924"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2448,7 +2448,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27111044"/>
+        <c:crossAx val="39755150"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2705,9 +2705,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>603000</xdr:colOff>
+      <xdr:colOff>602640</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>182160</xdr:rowOff>
+      <xdr:rowOff>181800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2716,7 +2716,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4883760" cy="3420720"/>
+        <a:ext cx="4883400" cy="3420360"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -8414,12 +8414,12 @@
         <v>318</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>319</v>
@@ -8434,40 +8434,40 @@
         <v>61</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H87" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I87" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J87" s="1" t="n">
         <v>0.2</v>
       </c>
-      <c r="I87" s="1" t="n">
+      <c r="K87" s="1" t="n">
         <v>0.15</v>
       </c>
-      <c r="J87" s="1" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K87" s="1" t="n">
-        <v>0.1</v>
-      </c>
       <c r="L87" s="1" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="M87" s="1" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="N87" s="1" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="O87" s="1" t="n">
         <f aca="false">H87*Methodology!$E$4+I87*Methodology!$E$5+J87*Methodology!$E$6+K87*Methodology!$E$7+L87*Methodology!$E$8+M87*Methodology!$E$9+N87*Methodology!$E$10</f>
-        <v>0.205</v>
+        <v>0.3175</v>
       </c>
       <c r="P87" s="1" t="n">
         <f aca="false">1+(O87*2.25)</f>
-        <v>1.46125</v>
+        <v>1.714375</v>
       </c>
       <c r="Q87" s="1" t="n">
         <f aca="false">ROUND(P87,0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R87" s="1" t="s">
         <v>321</v>
@@ -8567,11 +8567,11 @@
       </c>
       <c r="C4" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A4)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A4,Evaluations!$P$2:$P$200)</f>
-        <v>1.219375</v>
+        <v>1.15890625</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8583,11 +8583,11 @@
       </c>
       <c r="C5" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A5)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A5,Evaluations!$P$2:$P$200)</f>
-        <v>1.88345588235294</v>
+        <v>1.8740625</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Willow (1988) to tier 2 (score 1.85)
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
+++ b/Fantasy_Grimdark_Scale_Fully_Scored.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="328">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale: Methodology</t>
   </si>
@@ -988,6 +988,15 @@
   </si>
   <si>
     <t xml:space="preserve">Corrected from an earlier tier-1 placement: the pervasive Halloween Town horror aesthetic (skeleton/monster designs throughout, Sally's repeated self-dismemberment, Oogie Boogie sadistically gambling with Santa's life, children traumatized by monstrous gifts) is a lot of visible, disturbing content for a film whose plot ultimately resolves safely — Explicit Darkness was underweighted the first time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Willow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ron Howard / George Lucas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Queen Bavmorda's decree to imprison every pregnant woman in her kingdom to prevent a prophesied downfall is genuinely severe institutional cruelty, and Airk dies in battle — but the comic-tinged transformation magic, Sorsha's clean redemption arc, and Bavmorda's almost ironic self-inflicted defeat keep the register close to Narnia and Castle in the Sky.</t>
   </si>
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale Summary</t>
@@ -2314,7 +2323,7 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>17</c:v>
@@ -2346,11 +2355,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="39755150"/>
-        <c:axId val="83895924"/>
+        <c:axId val="51503892"/>
+        <c:axId val="91564592"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="39755150"/>
+        <c:axId val="51503892"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2395,7 +2404,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83895924"/>
+        <c:crossAx val="91564592"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2403,7 +2412,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="83895924"/>
+        <c:axId val="91564592"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2448,7 +2457,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39755150"/>
+        <c:crossAx val="51503892"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2705,9 +2714,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>602640</xdr:colOff>
+      <xdr:colOff>602280</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>181800</xdr:rowOff>
+      <xdr:rowOff>181440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2716,7 +2725,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7518960" y="438120"/>
-        <a:ext cx="4883400" cy="3420360"/>
+        <a:ext cx="4883040" cy="3420000"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3329,7 +3338,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R87"/>
+  <dimension ref="A1:R88"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -8471,6 +8480,65 @@
       </c>
       <c r="R87" s="1" t="s">
         <v>321</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H88" s="1" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I88" s="1" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J88" s="1" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K88" s="1" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="L88" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M88" s="1" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N88" s="1" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="O88" s="1" t="n">
+        <f aca="false">H88*Methodology!$E$4+I88*Methodology!$E$5+J88*Methodology!$E$6+K88*Methodology!$E$7+L88*Methodology!$E$8+M88*Methodology!$E$9+N88*Methodology!$E$10</f>
+        <v>0.3775</v>
+      </c>
+      <c r="P88" s="1" t="n">
+        <f aca="false">1+(O88*2.25)</f>
+        <v>1.849375</v>
+      </c>
+      <c r="Q88" s="1" t="n">
+        <f aca="false">ROUND(P88,0)</f>
+        <v>2</v>
+      </c>
+      <c r="R88" s="1" t="s">
+        <v>324</v>
       </c>
     </row>
   </sheetData>
@@ -8536,7 +8604,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -8552,10 +8620,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8583,11 +8651,11 @@
       </c>
       <c r="C5" s="1" t="n">
         <f aca="false">COUNTIF(Evaluations!$A$2:$A$200,A5)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D5" s="11" t="n">
         <f aca="false">AVERAGEIF(Evaluations!$A$2:$A$200,A5,Evaluations!$P$2:$P$200)</f>
-        <v>1.8740625</v>
+        <v>1.87276315789474</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>